<commit_message>
Update Energy Administration API data
</commit_message>
<xml_diff>
--- a/output/zone_monthly_3_02/electricity_generation_3_02.xlsx
+++ b/output/zone_monthly_3_02/electricity_generation_3_02.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="monthly" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="annual" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="data_dictionary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10165,4 +10166,958 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>column_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>original_column</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>source_section</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>資料區塊名稱</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>例如：全國、台電、民營電廠、自用發電設備</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>roc_period</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>民國年/月期間</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>各區塊第一欄</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>例如：114年、01月、115年01-03月</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>period</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>西元期間</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Column29 / Column26 / Column20 等</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>monthly 為 YYYY/MM；annual 為 YYYY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>total_gwh</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>發電量總計</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>total_share_pct</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>發電量總計占比</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>全國區塊通常沒有此欄；台電、民營電廠等區塊可能有</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>pumped_storage_gwh</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>抽蓄水力發電量</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>pumped_storage_share_pct</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>抽蓄水力發電占比</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>thermal_total_gwh</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>火力發電合計</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>thermal_total_share_pct</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>火力發電合計占比</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>coal_gwh</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>燃煤發電量</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>coal_share_pct</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>燃煤發電占比</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>oil_gwh</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>燃油發電量</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>民營電廠區塊可能沒有此欄</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>oil_share_pct</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>燃油發電占比</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>民營電廠區塊可能沒有此欄</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>lng_gwh</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>燃氣發電量</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>原始表頭為燃氣 / LNG-Fired</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>lng_share_pct</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>燃氣發電占比</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>原始表頭為燃氣 / LNG-Fired</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nuclear_gwh</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>核能發電量</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nuclear_share_pct</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>核能發電占比</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>renewable_total_gwh</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>再生能源發電合計</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>renewable_total_share_pct</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>再生能源發電合計占比</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>hydro_gwh</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>慣常水力發電量</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>hydro_share_pct</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>慣常水力發電占比</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>geothermal_gwh</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>地熱發電量</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>geothermal_share_pct</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>地熱發電占比</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>solar_pv_gwh</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>太陽光電發電量</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>solar_pv_share_pct</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>太陽光電發電占比</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>wind_gwh</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>風力發電量</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>原始資料註記：風力統計自 111 年 1 月起納入併聯試運轉發電量，部分月份可能波動較大</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>wind_share_pct</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>風力發電占比</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>原始資料註記：風力統計自 111 年 1 月起納入併聯試運轉發電量，部分月份可能波動較大</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>biomass_gwh</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>生質能發電量</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>部分區塊可能沒有此欄</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>biomass_share_pct</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>生質能發電占比</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>部分區塊可能沒有此欄</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>waste_gwh</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>廢棄物發電量</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>GWh</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>部分區塊可能沒有此欄</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>monthly / annual</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>waste_share_pct</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>廢棄物發電占比</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>依 source_section 而異</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>部分區塊可能沒有此欄</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>